<commit_message>
frontend 2nd move to public
</commit_message>
<xml_diff>
--- a/public/tutorial/tutorial_steps_full_complete.xlsx
+++ b/public/tutorial/tutorial_steps_full_complete.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\82109\Documents\My Lab\4_My Factory\CodingNDeveloping\웹코딩\Ltryi_Frontend_moved\LTsRYI\tutorial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE95E575-19BE-448B-9D05-480D9A36C5AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{050F7D4B-DA17-4537-BA9F-49366C333A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1260" yWindow="1440" windowWidth="14880" windowHeight="11060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39345" yWindow="8130" windowWidth="14880" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -214,9 +214,6 @@
     <t>반납함입니다.</t>
   </si>
   <si>
-    <t>이렇게 숙제 전송까지 완료되었어요!</t>
-  </si>
-  <si>
     <t>highlight</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -419,14 +416,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>300_80_280_90</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>310_155_200_90</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>숙제 하나 완료!
 Level Test도 똑같이 
 완료해볼까요?</t>
@@ -481,12 +470,6 @@
   </si>
   <si>
     <t>290_10_270_100</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">첫번째 메뉴에서는 
-당신의 현재 진척도를 체크하고, 
-추천 숙제를 받아보세요. </t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -580,11 +563,6 @@
   <si>
     <t xml:space="preserve">자유롭게 
 아래 메뉴를 눌러보세요.                 </t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>그 사이, 전송이 완료됐대요! 
-다시 카페 홀로 나가볼까요!</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -681,8 +659,14 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>480_50_200_90</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <r>
-      <t xml:space="preserve">작성을 다 끝내셨다면, </t>
+      <t xml:space="preserve">작성을 다 끝내셨다면,
+‘완료했어요’ 버튼을 눌러서 
+완료 표시를 해보세요! </t>
     </r>
     <r>
       <rPr>
@@ -691,20 +675,28 @@
         <rFont val="Segoe UI Symbol"/>
         <family val="2"/>
       </rPr>
-      <t>⬆</t>
+      <t>⬇</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-‘완료했어요’ 버튼을 눌러서 
-완료 표시를 해보세요!</t>
-    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>360_155_200_90</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>전송도 끄읕!
+이렇게 숙제 전송까지 완료되었어요!</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">첫번째 메뉴에서는 
+당신의 현재 진도를 체크하고, 
+추천 숙제를 받아보세요. </t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>아참, 전송은 완료됐대요. 
+둘러보시다가, 점수 보러!</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1155,7 +1147,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
@@ -1193,7 +1185,7 @@
         <v>13</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="G3" t="s">
         <v>56</v>
@@ -1213,7 +1205,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="G4" t="s">
         <v>56</v>
@@ -1233,13 +1225,13 @@
         <v>15</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="G5" t="s">
         <v>56</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="51" x14ac:dyDescent="0.45">
@@ -1256,13 +1248,13 @@
         <v>16</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="G6" t="s">
         <v>56</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="34" x14ac:dyDescent="0.45">
@@ -1276,7 +1268,7 @@
         <v>17</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F7" t="s">
         <v>52</v>
@@ -1285,7 +1277,7 @@
         <v>59</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.45">
@@ -1299,13 +1291,13 @@
         <v>18</v>
       </c>
       <c r="E8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F8" t="s">
         <v>58</v>
       </c>
       <c r="G8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="34" x14ac:dyDescent="0.45">
@@ -1319,16 +1311,16 @@
         <v>19</v>
       </c>
       <c r="E9" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F9" t="s">
+        <v>66</v>
+      </c>
+      <c r="G9" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>102</v>
-      </c>
-      <c r="F9" t="s">
-        <v>67</v>
-      </c>
-      <c r="G9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.45">
@@ -1342,16 +1334,16 @@
         <v>20</v>
       </c>
       <c r="E10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="F10" t="s">
-        <v>68</v>
-      </c>
-      <c r="G10" t="s">
-        <v>56</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="51" x14ac:dyDescent="0.45">
@@ -1365,16 +1357,16 @@
         <v>21</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F11" t="s">
         <v>58</v>
       </c>
       <c r="G11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.45">
@@ -1391,13 +1383,13 @@
         <v>50</v>
       </c>
       <c r="F12" t="s">
+        <v>71</v>
+      </c>
+      <c r="G12" t="s">
         <v>72</v>
       </c>
-      <c r="G12" t="s">
-        <v>73</v>
-      </c>
       <c r="H12" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.45">
@@ -1405,19 +1397,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D13" t="s">
         <v>23</v>
       </c>
       <c r="E13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" t="s">
         <v>69</v>
       </c>
-      <c r="F13" t="s">
-        <v>70</v>
-      </c>
       <c r="G13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="34" x14ac:dyDescent="0.45">
@@ -1431,7 +1423,7 @@
         <v>24</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="F14" t="s">
         <v>53</v>
@@ -1440,7 +1432,7 @@
         <v>56</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="51" x14ac:dyDescent="0.45">
@@ -1454,16 +1446,16 @@
         <v>25</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F15" t="s">
         <v>60</v>
       </c>
       <c r="G15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.45">
@@ -1471,7 +1463,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C16" t="s">
         <v>10</v>
@@ -1483,7 +1475,7 @@
         <v>51</v>
       </c>
       <c r="G16" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="68" x14ac:dyDescent="0.45">
@@ -1497,13 +1489,13 @@
         <v>27</v>
       </c>
       <c r="E17" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="G17" t="s">
+        <v>73</v>
+      </c>
+      <c r="H17" s="5" t="s">
         <v>110</v>
-      </c>
-      <c r="G17" t="s">
-        <v>74</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="51" x14ac:dyDescent="0.45">
@@ -1517,16 +1509,16 @@
         <v>28</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="F18" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>112</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="51" x14ac:dyDescent="0.45">
@@ -1540,16 +1532,16 @@
         <v>29</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="F19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>113</v>
+        <v>160</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="51" x14ac:dyDescent="0.45">
@@ -1563,13 +1555,13 @@
         <v>30</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="68" x14ac:dyDescent="0.45">
@@ -1586,7 +1578,7 @@
         <v>31</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G21" t="s">
         <v>56</v>
@@ -1597,19 +1589,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="F22" t="s">
+        <v>77</v>
+      </c>
+      <c r="G22" t="s">
         <v>78</v>
       </c>
-      <c r="G22" t="s">
-        <v>79</v>
-      </c>
       <c r="H22" s="5" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.45">
@@ -1617,7 +1609,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>61</v>
@@ -1631,19 +1623,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F24" t="s">
+        <v>79</v>
+      </c>
+      <c r="G24" t="s">
         <v>80</v>
       </c>
-      <c r="G24" t="s">
-        <v>81</v>
-      </c>
       <c r="H24" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="34" x14ac:dyDescent="0.45">
@@ -1651,30 +1643,30 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="F25" t="s">
+        <v>81</v>
+      </c>
+      <c r="G25" t="s">
         <v>82</v>
       </c>
-      <c r="G25" t="s">
-        <v>83</v>
-      </c>
       <c r="H25" s="5" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.45">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="51" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
         <v>57</v>
       </c>
-      <c r="E26" s="3" t="s">
-        <v>62</v>
+      <c r="E26" s="7" t="s">
+        <v>161</v>
       </c>
       <c r="G26" t="s">
         <v>56</v>
@@ -1688,7 +1680,7 @@
         <v>57</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G27" t="s">
         <v>56</v>
@@ -1702,7 +1694,7 @@
         <v>57</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="G28" t="s">
         <v>56</v>
@@ -1713,19 +1705,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F29" t="s">
+        <v>89</v>
+      </c>
+      <c r="G29" t="s">
         <v>90</v>
       </c>
-      <c r="G29" t="s">
-        <v>91</v>
-      </c>
       <c r="H29" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="51" x14ac:dyDescent="0.45">
@@ -1733,16 +1725,16 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G30" t="s">
         <v>56</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="51" x14ac:dyDescent="0.45">
@@ -1750,22 +1742,22 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D31" t="s">
         <v>32</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>125</v>
+        <v>162</v>
       </c>
       <c r="F31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G31" t="s">
         <v>56</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="34" x14ac:dyDescent="0.45">
@@ -1773,22 +1765,22 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D32" t="s">
         <v>33</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G32" t="s">
         <v>56</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="34" x14ac:dyDescent="0.45">
@@ -1796,19 +1788,19 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D33" t="s">
         <v>34</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="G33" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="34" x14ac:dyDescent="0.45">
@@ -1816,16 +1808,16 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D34" t="s">
         <v>35</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="68" x14ac:dyDescent="0.45">
@@ -1839,16 +1831,16 @@
         <v>36</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="F35" t="s">
+        <v>85</v>
+      </c>
+      <c r="G35" t="s">
         <v>86</v>
       </c>
-      <c r="G35" t="s">
-        <v>87</v>
-      </c>
       <c r="H35" s="5" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="51" x14ac:dyDescent="0.45">
@@ -1856,19 +1848,19 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D36" t="s">
         <v>37</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="G36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="85" x14ac:dyDescent="0.45">
@@ -1882,16 +1874,16 @@
         <v>38</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F37" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G37" t="s">
         <v>56</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="51" x14ac:dyDescent="0.45">
@@ -1905,16 +1897,16 @@
         <v>39</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="F38" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G38" t="s">
         <v>56</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.45">
@@ -1922,7 +1914,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C39" t="s">
         <v>11</v>
@@ -1931,7 +1923,7 @@
         <v>40</v>
       </c>
       <c r="E39" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="G39" t="s">
         <v>56</v>
@@ -1951,7 +1943,7 @@
         <v>41</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="G40" t="s">
         <v>56</v>
@@ -1962,19 +1954,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D41" t="s">
         <v>42</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="G41" t="s">
         <v>56</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="68" x14ac:dyDescent="0.45">
@@ -1991,7 +1983,7 @@
         <v>43</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="G42" t="s">
         <v>56</v>
@@ -2011,7 +2003,7 @@
         <v>44</v>
       </c>
       <c r="E43" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G43" t="s">
         <v>56</v>
@@ -2031,7 +2023,7 @@
         <v>45</v>
       </c>
       <c r="E44" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G44" t="s">
         <v>56</v>
@@ -2051,7 +2043,7 @@
         <v>46</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F45" t="s">
         <v>54</v>
@@ -2074,7 +2066,7 @@
         <v>47</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="F46" t="s">
         <v>55</v>
@@ -2097,7 +2089,7 @@
         <v>48</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G47" t="s">
         <v>56</v>
@@ -2111,10 +2103,10 @@
         <v>7</v>
       </c>
       <c r="C48" t="s">
+        <v>64</v>
+      </c>
+      <c r="E48" t="s">
         <v>65</v>
-      </c>
-      <c r="E48" t="s">
-        <v>66</v>
       </c>
       <c r="G48" t="s">
         <v>56</v>

</xml_diff>